<commit_message>
Confirm accurate xlsx and csv files for birch_2026-05-05
</commit_message>
<xml_diff>
--- a/tests/fixtures/birch_2026-05-05/runsetup.xlsx
+++ b/tests/fixtures/birch_2026-05-05/runsetup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bhanke\Projects\comact-runsetup-translator\tests\fixtures\birch_2026-05-05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{1CCD8B6A-1341-413B-9764-05E3347ED279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BFF514E4-CCD0-428D-96D5-90BB4ED82284}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29580" yWindow="-4785" windowWidth="11625" windowHeight="15390" xr2:uid="{E094D080-3319-4F65-806B-502944EB452C}"/>
+    <workbookView xWindow="4110" yWindow="615" windowWidth="22500" windowHeight="15390" xr2:uid="{E094D080-3319-4F65-806B-502944EB452C}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>